<commit_message>
before pulling extent report
</commit_message>
<xml_diff>
--- a/Languages.xlsx
+++ b/Languages.xlsx
@@ -12,35 +12,65 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="115">
+  <si>
+    <t>Language</t>
+  </si>
+  <si>
+    <t>Language Count</t>
+  </si>
   <si>
     <t>English</t>
   </si>
   <si>
+    <t>260</t>
+  </si>
+  <si>
     <t>Spanish</t>
   </si>
   <si>
+    <t>202</t>
+  </si>
+  <si>
     <t>Chinese</t>
   </si>
   <si>
+    <t>195</t>
+  </si>
+  <si>
     <t>French</t>
   </si>
   <si>
+    <t>188</t>
+  </si>
+  <si>
     <t>Pushto</t>
   </si>
   <si>
+    <t>186</t>
+  </si>
+  <si>
     <t>Portuguese</t>
   </si>
   <si>
+    <t>184</t>
+  </si>
+  <si>
     <t>Arabic</t>
   </si>
   <si>
+    <t>183</t>
+  </si>
+  <si>
     <t>German</t>
   </si>
   <si>
     <t>Hindi</t>
   </si>
   <si>
+    <t>181</t>
+  </si>
+  <si>
     <t>Indonesian</t>
   </si>
   <si>
@@ -50,18 +80,30 @@
     <t>Japanese</t>
   </si>
   <si>
+    <t>171</t>
+  </si>
+  <si>
     <t>Korean</t>
   </si>
   <si>
     <t>Italian</t>
   </si>
   <si>
+    <t>169</t>
+  </si>
+  <si>
     <t>Swedish</t>
   </si>
   <si>
+    <t>168</t>
+  </si>
+  <si>
     <t>Dutch</t>
   </si>
   <si>
+    <t>167</t>
+  </si>
+  <si>
     <t>Greek</t>
   </si>
   <si>
@@ -83,48 +125,90 @@
     <t>Azerbaijani</t>
   </si>
   <si>
+    <t>126</t>
+  </si>
+  <si>
     <t>Vietnamese</t>
   </si>
   <si>
+    <t>124</t>
+  </si>
+  <si>
     <t>Hungarian</t>
   </si>
   <si>
+    <t>116</t>
+  </si>
+  <si>
     <t>Urdu</t>
   </si>
   <si>
+    <t>115</t>
+  </si>
+  <si>
     <t>Bengali</t>
   </si>
   <si>
+    <t>111</t>
+  </si>
+  <si>
     <t>Persian</t>
   </si>
   <si>
+    <t>23</t>
+  </si>
+  <si>
     <t>Uzbek</t>
   </si>
   <si>
+    <t>18</t>
+  </si>
+  <si>
     <t>Afrikaans</t>
   </si>
   <si>
+    <t>16</t>
+  </si>
+  <si>
     <t>Oriya</t>
   </si>
   <si>
+    <t>9</t>
+  </si>
+  <si>
     <t>Mongolian</t>
   </si>
   <si>
+    <t>7</t>
+  </si>
+  <si>
     <t>Catalan</t>
   </si>
   <si>
+    <t>6</t>
+  </si>
+  <si>
     <t>Slovak</t>
   </si>
   <si>
+    <t>5</t>
+  </si>
+  <si>
     <t>Tamil</t>
   </si>
   <si>
     <t>Serbian</t>
   </si>
   <si>
+    <t>4</t>
+  </si>
+  <si>
     <t>Czech</t>
   </si>
   <si>
+    <t>3</t>
+  </si>
+  <si>
     <t>Hebrew</t>
   </si>
   <si>
@@ -137,6 +221,9 @@
     <t>Albanian</t>
   </si>
   <si>
+    <t>2</t>
+  </si>
+  <si>
     <t>Burmese</t>
   </si>
   <si>
@@ -149,6 +236,9 @@
     <t>Bulgarian</t>
   </si>
   <si>
+    <t>1</t>
+  </si>
+  <si>
     <t>Croatian</t>
   </si>
   <si>
@@ -159,6 +249,114 @@
   </si>
   <si>
     <t>Swahili</t>
+  </si>
+  <si>
+    <t>Courses</t>
+  </si>
+  <si>
+    <t>254</t>
+  </si>
+  <si>
+    <t>Specializations</t>
+  </si>
+  <si>
+    <t>42</t>
+  </si>
+  <si>
+    <t>Professional Certificates</t>
+  </si>
+  <si>
+    <t>Beginner</t>
+  </si>
+  <si>
+    <t>120</t>
+  </si>
+  <si>
+    <t>Intermediate</t>
+  </si>
+  <si>
+    <t>104</t>
+  </si>
+  <si>
+    <t>Advanced</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>Mixed</t>
+  </si>
+  <si>
+    <t>53</t>
+  </si>
+  <si>
+    <t>1-4 Weeks</t>
+  </si>
+  <si>
+    <t>94</t>
+  </si>
+  <si>
+    <t>1-3 Months</t>
+  </si>
+  <si>
+    <t>170</t>
+  </si>
+  <si>
+    <t>3-6 Months</t>
+  </si>
+  <si>
+    <t>33</t>
+  </si>
+  <si>
+    <t>English Language</t>
+  </si>
+  <si>
+    <t>Language Learning</t>
+  </si>
+  <si>
+    <t>Language Competency</t>
+  </si>
+  <si>
+    <t>177</t>
+  </si>
+  <si>
+    <t>Vocabulary</t>
+  </si>
+  <si>
+    <t>176</t>
+  </si>
+  <si>
+    <t>Arizona State University</t>
+  </si>
+  <si>
+    <t>61</t>
+  </si>
+  <si>
+    <t>University of California, Irvine</t>
+  </si>
+  <si>
+    <t>Voxy</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>Peking University</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>Dialogues And Role Plays</t>
+  </si>
+  <si>
+    <t>Coding Labs</t>
+  </si>
+  <si>
+    <t>ChatGPT</t>
+  </si>
+  <si>
+    <t>Google Gemini</t>
   </si>
 </sst>
 </file>
@@ -203,252 +401,619 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A49"/>
+  <dimension ref="A1:B76"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="24.7109375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="13.8359375" customWidth="true" bestFit="true"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
+      <c r="B1" t="s" s="0">
+        <v>1</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>3</v>
+        <v>6</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>4</v>
+        <v>8</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>5</v>
+        <v>10</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>11</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>6</v>
+        <v>12</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>13</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>7</v>
+        <v>14</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>15</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>8</v>
+        <v>16</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>15</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>9</v>
+        <v>17</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>18</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>10</v>
+        <v>19</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>18</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>11</v>
+        <v>20</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>18</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>12</v>
+        <v>21</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>22</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>13</v>
+        <v>23</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>22</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>14</v>
+        <v>24</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>25</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>15</v>
+        <v>26</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>27</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>16</v>
+        <v>28</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>17</v>
+        <v>30</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>18</v>
+        <v>31</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>19</v>
+        <v>32</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>20</v>
+        <v>33</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>21</v>
+        <v>34</v>
+      </c>
+      <c r="B22" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>22</v>
+        <v>35</v>
+      </c>
+      <c r="B23" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>23</v>
+        <v>36</v>
+      </c>
+      <c r="B24" t="s" s="0">
+        <v>37</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>24</v>
+        <v>38</v>
+      </c>
+      <c r="B25" t="s" s="0">
+        <v>39</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>25</v>
+        <v>40</v>
+      </c>
+      <c r="B26" t="s" s="0">
+        <v>41</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>26</v>
+        <v>42</v>
+      </c>
+      <c r="B27" t="s" s="0">
+        <v>43</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>27</v>
+        <v>44</v>
+      </c>
+      <c r="B28" t="s" s="0">
+        <v>45</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>28</v>
+        <v>46</v>
+      </c>
+      <c r="B29" t="s" s="0">
+        <v>47</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>29</v>
+        <v>48</v>
+      </c>
+      <c r="B30" t="s" s="0">
+        <v>49</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>30</v>
+        <v>50</v>
+      </c>
+      <c r="B31" t="s" s="0">
+        <v>51</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
-        <v>31</v>
+        <v>52</v>
+      </c>
+      <c r="B32" t="s" s="0">
+        <v>53</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>32</v>
+        <v>54</v>
+      </c>
+      <c r="B33" t="s" s="0">
+        <v>55</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="0">
-        <v>33</v>
+        <v>56</v>
+      </c>
+      <c r="B34" t="s" s="0">
+        <v>57</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="0">
-        <v>34</v>
+        <v>58</v>
+      </c>
+      <c r="B35" t="s" s="0">
+        <v>59</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="0">
-        <v>35</v>
+        <v>60</v>
+      </c>
+      <c r="B36" t="s" s="0">
+        <v>59</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="0">
-        <v>36</v>
+        <v>61</v>
+      </c>
+      <c r="B37" t="s" s="0">
+        <v>62</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="0">
-        <v>37</v>
+        <v>63</v>
+      </c>
+      <c r="B38" t="s" s="0">
+        <v>64</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="0">
-        <v>38</v>
+        <v>65</v>
+      </c>
+      <c r="B39" t="s" s="0">
+        <v>64</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="0">
-        <v>39</v>
+        <v>66</v>
+      </c>
+      <c r="B40" t="s" s="0">
+        <v>64</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="0">
-        <v>40</v>
+        <v>67</v>
+      </c>
+      <c r="B41" t="s" s="0">
+        <v>64</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="0">
-        <v>41</v>
+        <v>68</v>
+      </c>
+      <c r="B42" t="s" s="0">
+        <v>69</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="0">
-        <v>42</v>
+        <v>70</v>
+      </c>
+      <c r="B43" t="s" s="0">
+        <v>69</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="0">
-        <v>43</v>
+        <v>71</v>
+      </c>
+      <c r="B44" t="s" s="0">
+        <v>69</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s" s="0">
-        <v>44</v>
+        <v>72</v>
+      </c>
+      <c r="B45" t="s" s="0">
+        <v>69</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s" s="0">
-        <v>45</v>
+        <v>73</v>
+      </c>
+      <c r="B46" t="s" s="0">
+        <v>74</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="0">
-        <v>46</v>
+        <v>75</v>
+      </c>
+      <c r="B47" t="s" s="0">
+        <v>74</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="0">
-        <v>47</v>
+        <v>76</v>
+      </c>
+      <c r="B48" t="s" s="0">
+        <v>74</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="0">
-        <v>48</v>
+        <v>77</v>
+      </c>
+      <c r="B49" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="B50" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="B51" t="s" s="0">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="B52" t="s" s="0">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s" s="0">
+        <v>83</v>
+      </c>
+      <c r="B53" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s" s="0">
+        <v>84</v>
+      </c>
+      <c r="B54" t="s" s="0">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="B55" t="s" s="0">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="B56" t="s" s="0">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="B57" t="s" s="0">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="B58" t="s" s="0">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s" s="0">
+        <v>94</v>
+      </c>
+      <c r="B59" t="s" s="0">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s" s="0">
+        <v>96</v>
+      </c>
+      <c r="B60" t="s" s="0">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="B61" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s" s="0">
+        <v>99</v>
+      </c>
+      <c r="B62" t="s" s="0">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s" s="0">
+        <v>100</v>
+      </c>
+      <c r="B63" t="s" s="0">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s" s="0">
+        <v>102</v>
+      </c>
+      <c r="B64" t="s" s="0">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="B65" t="s" s="0">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="B66" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B67" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="B68" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s" s="0">
+        <v>104</v>
+      </c>
+      <c r="B69" t="s" s="0">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s" s="0">
+        <v>106</v>
+      </c>
+      <c r="B70" t="s" s="0">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="s" s="0">
+        <v>107</v>
+      </c>
+      <c r="B71" t="s" s="0">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="s" s="0">
+        <v>109</v>
+      </c>
+      <c r="B72" t="s" s="0">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="s" s="0">
+        <v>111</v>
+      </c>
+      <c r="B73" t="s" s="0">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="s" s="0">
+        <v>112</v>
+      </c>
+      <c r="B74" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="s" s="0">
+        <v>113</v>
+      </c>
+      <c r="B75" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="B76" t="s" s="0">
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>